<commit_message>
jp_delivery 01 要件定義書 v1.1-draft 収尾コミット — IPA 9 構成再整理 (DRAFT)
in-flight (2026-05-13 起草) の未コミット改動を確定. v1.1 正式版 PASS ではない.

- 構造: v1.0 (6 節) → IPA 要件定義書 標準準拠 9 構成
  (背景 / 業務上の課題 / 目標利用者 / 業務要件 / 機能要件 / 非機能要件 / 採用原則 / 制約条件 / 前提条件)
- 実装レベル記述を 02 基本設計書 + 04 テスト結果報告書へ移行
- 日本語表記を CDISC 業界用法 (規格 / コントロールド・ターミノロジー 等) に統一
- 機械検証: yaml parse OK + xlsx↔yml mtime 一致 + audit_terms blacklist hits=0 PASS
- DRAFT 状態: PASS 五条 第2条(形式)+第4条(用語監査) のみ達成;
  第3条 reviewer round + 第5条 用户 ack は未実施 (用户「只看现状不开工」選択)
- Chain J/B 双写: CHANGELOG + _progress.json (v1_1_draft 追加, v1.0 PASS 記録保持)
  + worklog/phase_jp_delivery.md + docs/PROGRESS.md (stale jp 行訂正)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/branches/jp_delivery/01_要件定義書.xlsx
+++ b/branches/jp_delivery/01_要件定義書.xlsx
@@ -10,25 +10,31 @@
     <sheet name="1_表紙" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2_改訂履歴" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3_目次" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="1_背景目的" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="2_業務要件" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="3_機能要件" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="4_非機能要件" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="5_制約条件" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="6_前提条件" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="4_承認欄" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="1_背景" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2_業務上の課題" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="3_目標利用者" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="4_業務要件" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="5_機能要件" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="6_非機能要件" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="7_採用原則" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="8_制約条件" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="9_前提条件" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="4_承認欄" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'1_表紙'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'2_改訂履歴'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'3_目次'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'1_背景目的'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'2_業務要件'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'3_機能要件'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'4_非機能要件'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'5_制約条件'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="8">'6_前提条件'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'4_承認欄'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'1_背景'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'2_業務上の課題'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'3_目標利用者'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'4_業務要件'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'5_機能要件'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'6_非機能要件'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'7_採用原則'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'8_制約条件'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'9_前提条件'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'4_承認欄'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -174,6 +180,9 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -206,9 +215,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -622,7 +628,7 @@
       <c r="A4" s="1" t="n"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>文書番号: ITMS-SDTM-01-REQUIREMENTS-DEFINITION-v1.0</t>
+          <t>文書番号: ITMS-SDTM-01-REQUIREMENTS-DEFINITION-v1.1-draft</t>
         </is>
       </c>
     </row>
@@ -671,7 +677,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-13</t>
         </is>
       </c>
     </row>
@@ -683,7 +689,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>v1.0</t>
+          <t>v1.1-draft</t>
         </is>
       </c>
     </row>
@@ -699,7 +705,7 @@
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -715,6 +721,358 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>7_採用原則</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>原則 ID</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>原則項目</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>原則内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>PR-01</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>規格優先性原則</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>本知識ベースは公式刊行物の代替ではなく業務参照のための再構成である。規格と差異が発生した場合は規格が優先される。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>PR-02</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>出典追跡可能性原則</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>本知識ベースに含まれる任意の記述は、原典 (公式刊行物の頁または節) まで追跡可能であること。出典のない主張は許容しない。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>PR-03</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>完全性志向原則</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>プレースホルダ (TBD 等) を完成版に残さない。未確定部分は要件として明示し、解消後に正式版に反映する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>PR-04</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>独立確認原則</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>本知識ベースの内容は、作成者と確認者を分離して品質を担保する。同一担当者による自己確認のみでの確定は許容しない。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+  <headerFooter>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>8_制約条件</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>制約 ID</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>種別</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>制約内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>C-01</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>著作権</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>SDTM、SDTMIG、CDISC Controlled Terminology の各規格および原刊行物の著作権は CDISC が保持する。本知識ベースは原刊行物そのものを再配布せず、業務参照用に再構成した派生著作物として、内部利用または公開ライセンス (CC BY 4.0 等) のもとでのみ配布する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>C-02</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>規制範囲外</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>本知識ベースは、米国 21 CFR Part 11 または PMDA 電子記録・電子署名指針が要求する電磁的記録の代替ではない。組標準作業手順書が当該電子記録を規定する場合、その規定が優先される。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>C-03</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>機密区分</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>本知識ベースおよび関連納品文書の機密区分は公開可レベルとする。CDISC 規格自体が公開資料であり、個人情報および組織機密情報を含めない。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+  <headerFooter>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>9_前提条件</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>前提 ID</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>種別</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>前提内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>P-01</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>一次資料利用可能性</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>利用者は、必要に応じて CDISC 公式刊行物 4 件 (SDTMIG v3.4 PDF / SDTM Model v2.0 PDF / SDTMIG xlsx v3.4 / Controlled Terminology xlsx 2024 年版) を CDISC Library 経由で参照可能であること。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>P-02</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>利用者背景</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>利用者は IT 分野および医療データ分野の双方に基本知識を有する実務担当者であること。基本的な臨床試験用語、Excel および Markdown の基本操作、業務関連規格への抵抗感のなさを想定する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>P-03</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>概念関係理解</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>利用者は SDTMIG v3.4 が SDTM Model v2.0 の実装ガイドである関係性を理解していること。SDTM Model v2.0 は概念モデル (観察クラス、変数役割、ドメイン分類体系) を規定し、SDTMIG v3.4 はこれを前提として各 Domain の具体実装を規定する。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>P-04</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>コントロールド・ターミノロジー体系理解</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>利用者は CDISC コントロールド・ターミノロジーの C コード体系 (例: C66731) を理解しており、米国国立がん研究所 EVS Browser (NCI EVS Browser) を用いたコード照合が可能であること。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+  <headerFooter>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -725,7 +1083,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>承認欄</t>
         </is>
@@ -790,7 +1148,7 @@
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -806,7 +1164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -859,11 +1217,33 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="16.5" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>v1.1-draft</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>構成を業界標準 (IPA 要件定義書) 準拠に再整理。背景・業務上の課題・目標利用者・業務要件・機能要件・非機能要件・採用原則・制約条件・前提条件の 9 構成に変更。実装記述は 02 基本設計書および 04 テスト結果報告書に移行。日本語表記を CDISC 業界用法 (規格 / コントロールド・ターミノロジー等) に統一。</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>張　泊江</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -879,7 +1259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -888,14 +1268,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>目次</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>(本文書のシート構成に合わせ自動生成)</t>
         </is>
@@ -920,170 +1300,221 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>1_表紙</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>表紙・文書情報</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>2_改訂履歴</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>版数・改訂内容の記録</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>3_目次</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>本シート</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>1_背景目的</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>本書の背景・目的・想定読者・関連文書</t>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>1_背景</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>業務の概要、SDTM 規格参照の業務上の位置付け、本書の範囲</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>2_業務要件</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>業務上の要件 — 本知識ベースが満たすべき業務的価値</t>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>2_業務上の課題</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>現状の SDTM 規格参照における業務上の課題と影響</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>3_機能要件</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>機能要件 — 工程別の構築機能と追跡機能</t>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>3_目標利用者</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>本知識ベースの主要利用者および副次利用者</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>4_非機能要件</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>非機能要件 — 品質・追跡可能性・規律統制</t>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>4_業務要件</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>業務上達成すべき要件</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>5_制約条件</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
-        <is>
-          <t>制約条件 — 本知識ベース利用時の前提となる制限事項</t>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>5_機能要件</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>業務要件を実現するために本知識ベースが具備すべき機能</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>6_前提条件</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>前提条件 — 利用環境・参照資料・読者前提知識</t>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>6_非機能要件</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>本知識ベースが満たすべき非機能特性</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>7_採用原則</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>本知識ベース構築および運用上の基本原則</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>8_制約条件</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>本知識ベースの構築および利用上の制約条件</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>9_前提条件</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>本知識ベース利用の前提条件</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>4_承認欄</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>作成・確認・承認の署名欄</t>
         </is>
@@ -1104,11 +1535,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1124,7 +1558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1133,163 +1567,114 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>1_背景目的</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>1_背景</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>1.1 本知識ベース (SDTM Knowledge Base) の存在意義</t>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>1.1 業務の概要</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="18" t="inlineStr">
-        <is>
-          <t>本知識ベースは、米国食品医薬品局 (FDA: Food and Drug Administration) が義務付け、独立行政法人医薬品医療機器総合機構 (PMDA: Pharmaceuticals and Medical Devices Agency) が認め、欧州医薬品庁 (EMA: European Medicines Agency) が受理する臨床試験データ表形式モデル (SDTM: Study Data Tabulation Model) の標準刊行物に基づき、業務利用しやすい形に再構成した参考資料である。</t>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>統合 G では、各臨床研究の電子データ収集 (EDC: Electronic Data Capture) システムから出力される CSV データを、CDISC 臨床試験データ表形式モデル (SDTM: Study Data Tabulation Model) の規格に従って変換する業務を担当している。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>対象は、CDISC SDTM 規格に依拠する臨床試験データ提出、データプログラミング、品質確認業務である。本知識ベースは、これら業務における日常参照を効率化することを目的とし、規制当局への提出時の権威源を代替するものではない。</t>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>本業務の遂行には、以下三領域の知識を統合的に参照する必要がある。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>1.2 本書の目的</t>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>・各研究の試験実施計画書 (Protocol)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>本書は、SDTM 知識ベース (SDTM Knowledge Base) が満たすべき要件を定義する。具体的には、業務要件 (§2)、機能要件 (§3)、非機能要件 (§4)、制約条件 (§5)、および前提条件 (§6) を体系的に記述し、iTMS 株式会社が本知識ベースの設計根拠・品質基準・利用上の前提を理解できるよう提示することを目的とする。</t>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>・臨床医療知識 (検査項目、診断、有害事象等)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>本知識ベースの設計・構成の詳細は 02 基本設計書に、日常運用手順は 03 運用保守マニュアルに、検証結果は 04 テスト結果報告書にそれぞれ委譲する。本書はこれら後続文書の共通根拠章であり、後続文書は本書の各節を引用して設計・運用・試験の根拠とする。</t>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>・SDTM 規格 (SDTMIG v3.4、SDTM Model v2.0、CDISC Controlled Terminology)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>1.3 想定読者</t>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>1.2 SDTM 規格参照の業務上の位置付け</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>本書の想定読者は、IT 分野および医療データ分野の双方に知見を有する実務担当者である。具体的には、臨床試験データ管理、SDTM データプログラミング、マッピング品質確認、SDTM 教育に従事する技術者および管理者を想定する。</t>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>CSV から SDTM への変換の各場面で、SDTM 規格への参照が発生する。具体的には以下の場面である。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>1.4 関連文書一覧</t>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>・Domain 判定: EDC 項目を SDTM の 63 ドメインのいずれに割り当てるかの判定。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>本書に関連する納品文書一覧は以下のとおりである。</t>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>・変数マッピング: SDTM 各変数の定義、Core 区分、許容値域への適合確認。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>・02 基本設計書: 本書の機能要件 (FR-01〜FR-11) および非機能要件 (NFR-01〜NFR-06) を実現する基本設計を提示する。</t>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>・コントロールド・ターミノロジー適用: 値が CDISC コントロールド・ターミノロジーのコードリストに整合するかの確認。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>・03 運用保守マニュアル: 本書の非機能要件 (NFR-04) および制約条件 (§5) に基づく日常運用手順・保守手順を記述する。</t>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>・業務前提確認: 各 Domain の業務上の前提 (Assumptions) との整合性確認。</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>・04 テスト結果報告書: 本書の前提条件 (§6) に基づき試験範囲を画定し、実施結果・合格判定・根拠資料を記録する。</t>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>これらの参照判断の精度と速度は、変換業務全体の生産性と品質に直接影響する。</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>・05 詳細設計書: 02 基本設計書の各章の詳細展開。</t>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>1.3 本書の範囲</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>・06 トレーサビリティ管理表: 本書の要件・設計・試験・根拠資料の横断対応表。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>・07 進捗報告書: 全体サマリ・工程別進捗・課題管理・今後の予定。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="C18" s="18" t="inlineStr">
-        <is>
-          <t>・99 用語集: 英語・日本語・中国語・出典規格の四列対照辞書。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>1.5 本書の位置付け</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>本書は、SDTM 知識ベースの要件を定義する最上位根拠文書である。後続三文書はそれぞれ本書の各節を引用して設計・運用・試験の根拠とする。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>・02 基本設計書は、本書 §3 機能要件 (FR-01〜FR-11) および §4 非機能要件 (NFR-01〜NFR-06) を実現する基本設計を提示する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>・03 運用保守マニュアルは、本書 §4 非機能要件および §5 制約条件に基づく運用手順を定める。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>・04 テスト結果報告書は、本書 §6 前提条件に従い試験範囲を画定する。</t>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>本書は、上記業務における SDTM 規格参照を効率化および高精度化するための社内利用知識ベース (以下「本知識ベース」) について、業務上必要となる要件を定義する。本書は要件のみを定義し、実装方式は別途 02 基本設計書および 05 詳細設計書において定める。</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1685,7 @@
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1316,7 +1701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -1325,121 +1710,142 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>2_業務要件</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>2_業務上の課題</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>2.1 業務シナリオ</t>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>2.1 SDTMIG v3.4 PDF 直接参照の負荷</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="18" t="inlineStr">
-        <is>
-          <t>本知識ベースは、以下三用途における作業参照資料として用いることを業務要件とする。</t>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>SDTMIG v3.4 公式刊行物は 461 頁の PDF として配布されており、業務担当者は必要時に該当部分を検索して参照している。しかし以下の負荷が日常的に発生している。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="18" t="inlineStr">
-        <is>
-          <t>・SDTM データプログラミング: 各ドメインの変数定義、Core 区分、受控用語との照合を日常参照する場面。</t>
+      <c r="C4" s="19" t="inlineStr">
+        <is>
+          <t>・任意の Domain、変数、用語の所在を特定するための時間的負荷 (461 頁の横断検索を要する)。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>・マッピング品質確認: 提出予定データセットを SDTMIG v3.4 仕様と照合し、不整合を抽出する場面。</t>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>・PDF の構造上、用語間の関連 (例: SUPPQUAL と他 Domain の関係) を辿る際に複数頁の往復が必要となる。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="18" t="inlineStr">
-        <is>
-          <t>・SDTM 教育: 規格初学者および中堅技術者が、ドメイン構造、観察クラス概念、受控用語体系を学習する場面。</t>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>・コントロールド・ターミノロジーは SDTMIG とは別の xlsx ファイルとして配布されており、PDF とのクロス参照が手作業となる。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>2.2 一次資料との対応関係</t>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>結果として、1 件の変数マッピング判断に対する規格参照に、数分から十数分を要する場面が生じる。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="C8" s="18" t="inlineStr">
-        <is>
-          <t>本知識ベースは、CDISC が公表する以下四種の公式刊行物のみを根拠とする。第三者要約や言換え版から派生したコンテンツを一切含まない。</t>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>2.2 既存 AI ツールによる参照の正答率問題</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>・SDTM 実装ガイド (SDTMIG: SDTM Implementation Guide) PDF v3.4 (2021 年 11 月 29 日公表)、461 頁。各ドメインの仕様、業務上の前提、実装例を収録する。</t>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>上記の PDF 参照負荷の代替手段として、業務担当者は一般的な AI ツール (汎用大規模言語モデルを用いた対話型サービス等) に SDTM 関連質問を投げる運用も試行している。しかし以下の問題がある。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>・SDTM モデル (SDTM Model) PDF v2.0 Final (2021 年 11 月 29 日公表)、74 頁。観察クラスおよび変数役割の概念モデルを規定する。</t>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>・回答の正答率が低く、SDTM 規格の実際の記述と異なる回答が頻繁に発生する。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>・SDTMIG xlsx v3.4。63 ドメインにわたる 1,917 変数の構造化メタデータを含む。</t>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>・出典 (公式刊行物の該当頁) が提示されず、回答の真偽確認が別途必要となる。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>・CDISC 受控用語 (Controlled Terminology) xlsx 2024 年版。1,005 のコードリスト、合計 37,939 用語を含む。</t>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>・推測値と規格記述が混在し、判断材料としての信頼性が確保できない。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>原刊行物自体は本リポジトリに再配布せず、CDISC が著作権を保持する。</t>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>・コントロールド・ターミノロジーのコード (例: C コード) の正確性が担保されない。</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>2.3 業務的限界</t>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>結果として、AI ツールの利用による効率化効果は限定的であり、最終的に PDF 直接参照に戻る場面が多い。</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>本知識ベースは作業参照資料としての性質を有し、以下二点の業務的限界を本書冒頭で明示する。</t>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>2.3 業務影響</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="C16" s="18" t="inlineStr">
-        <is>
-          <t>第一に、本知識ベースは、米国 21 CFR Part 11 または PMDA が想定する電子記録および電子署名要件を充足する電磁的記録の代替ではない。組織標準作業手順書がこれら電子記録について規定する場合、その規定が優先される。</t>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>上記 2.1 および 2.2 により、以下の業務影響が発生している。</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="C17" s="18" t="inlineStr">
-        <is>
-          <t>第二に、規制当局への提出時の権威源は CDISC 公式刊行物であり、本知識ベースの記述と公式刊行物との間に差異が見られた場合は、公式刊行物が優先される。</t>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>・変換業務における規格参照工数の累積的増大。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>・判断の確度の低下 (回答が規格に整合しているかを別途確認しないと信頼できない)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>・新規担当者の習熟期間の延長 (461 頁の PDF を体系的に学習する負担)。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>・組内での参照経験の属人化 (個別担当者の探索ノウハウが暗黙知化する)。</t>
         </is>
       </c>
     </row>
@@ -1450,7 +1856,7 @@
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1466,222 +1872,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="2" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>3_機能要件</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>要件 ID</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>要件項目</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>要件内容</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>3_目標利用者</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>3.1 主要利用者</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>FR-01</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>仕様自動変換機能</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>SDTMIG xlsx v3.4 を入力とし、63 ドメインの仕様 Markdown ファイルおよび用語索引を Python 処理単位で機械的に生成する。</t>
+      <c r="C3" s="19" t="inlineStr">
+        <is>
+          <t>統合 G および将来的に同等業務を担当する社員。具体的には以下の役割を想定する。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>FR-02</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>PDF ページ索引機能</t>
-        </is>
-      </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>SDTMIG v3.4 PDF を入力とし、ページ位置を機械的に索引化する。視覚的推定値を排除し、機械処理による精確なページ索引を唯一の参照源とする。</t>
+          <t>・SDTM 変換業務担当: EDC 出力 CSV から SDTM への変換を主に担当する者。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>FR-03</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>PDF 抽出機能</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>SDTMIG v3.4 PDF から各ドメインの業務上の前提および実装例を AI 補助で抽出する。全 11 処理単位に分割し、各処理単位ごとに独立確認を実施する。</t>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>・SDTM 品質確認担当: 変換結果の規格整合性を確認する者。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>FR-04</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>補完抽出機能</t>
-        </is>
-      </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>SDTM Model v2.0 PDF からモデル概念 6 文書、SDTMIG v3.4 PDF から共通章 6 文書を補完抽出する。</t>
+          <t>主要利用者は以下の前提知識を有することを想定する。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>FR-05</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>全件確認・索引化機能</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>全ファイルを対象に網羅確認を実施し、索引文書 INDEX.md を生成する。確認報告書を併せて産出する。</t>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>・臨床試験データ管理業務の基本知識。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>FR-06</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>検索最適化機能</t>
-        </is>
-      </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>経路層文書 ROUTING.md および逆引き変数索引 VARIABLE_INDEX.md (1,523 変数収録) を生成し、知識ベースの検索効率を向上させる。</t>
+          <t>・SDTM の基本概念 (Domain、変数、Core 区分、Controlled Terminology)。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>FR-07</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>AI 平台展開機能</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>知識ベースを四種の AI 平台向け配布物として整形する。各平台の容量制約および機能制約に整合させた構成で出力する。</t>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>・業務関連規格に対する抵抗感のないこと。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>FR-08</t>
-        </is>
-      </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>ドメイン回答追跡機能</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>ドメインに関する任意の主張について、ドメイン符号特定、knowledge_base/domains/&lt;DOMAIN&gt;/ 配下三件 (spec.md / assumptions.md / examples.md) の参照、PDF 頁範囲の照合の手順で、一次資料に追跡可能とする。</t>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>3.2 副次利用者</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>FR-09</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>章節回答追跡機能</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>章節レベルの主張について、knowledge_base/chapters/chXX_*.md の頁範囲および節番号が、SDTMIG 目次と直接対応する構造を提供する。</t>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>主要利用者に加え、以下の副次利用者も想定する。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>FR-10</t>
-        </is>
-      </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>受控用語追跡機能</t>
-        </is>
-      </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
-          <t>knowledge_base/terminology/ 配下の各コードリスト文書に CDISC 割当の C 符号 (例 C66731) を保持し、米国国立がん研究所 EVS Browser (NCI EVS Browser) との相互参照を可能とする。</t>
+          <t>・SDTM 学習者: SDTM 規格を初めて学習する新規担当者または異動者。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>FR-11</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>字面級確認継続実施機能</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>七工程パイプラインと並行し、知識ベースの字面級確認を独立した作業群として継続実施する。各検証単位の主張を出典 PDF と頁単位で照合する。2026 年 4 月 29 日時点で対象範囲の 97% を完了し、進行中である。</t>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>・教育担当: 統合 G 内での SDTM 教育を実施する担当者。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>・関連業務組: 将来的に SDTM 規格参照が必要となる他組のメンバー。</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1985,7 @@
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1708,184 +2001,114 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>4_非機能要件</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>4_業務要件</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>要件 ID</t>
+          <t>業務要件 ID</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>観点</t>
+          <t>要件項目</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
           <t>要件内容</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>ALCOA+ 次元</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>NFR-01</t>
+          <t>BR-01</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>定量合格判定基準</t>
+          <t>規格の即時参照</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>合格判定基準は定量化する。原典資料に対する覆盖率は 95% 以上、未記入・未確定マーカーは 0 件とする。主観的評価のみによる合格判定は許容しない。</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Complete · Accurate</t>
+          <t>業務担当者が SDTM 変換業務遂行中の任意の場面において、SDTM 規格の該当部分を数十秒以内に参照可能であること。任意の Domain の定義および変数一覧、任意の変数の定義および許容値、任意のコントロールド・ターミノロジーのコードリストを含む。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>NFR-02</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>作成者・承認者分離</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="inlineStr">
-        <is>
-          <t>コンテンツを作成した担当者は、当該コンテンツを承認できない。承認担当者は出典 PDF を独立に参照し、構造化された確認報告を作成する。</t>
-        </is>
-      </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>Attributable</t>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>BR-02</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>原典追跡</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>参照内容について、公式刊行物 (SDTMIG v3.4 PDF 等) の該当頁・節への追跡が常に可能であること。出典の付与されていない情報は許容しない。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>NFR-03</t>
+          <t>BR-03</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>AI 推測値の明示</t>
+          <t>AI 経由での高精度応答</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>AI が機械的に確認できない値はすべて (estimated) ラベルを付与する。当該値は権威索引から除外する。精確値が必要な場合は機械処理または人手照合を経る。なお (estimated) は知識ベース内部の機械可読ラベルとして英語表記のまま運用する。</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Original · Accurate</t>
+          <t>業務担当者が AI ツール経由で SDTM 関連質問を行った場合に、規格記述に整合した高精度な応答が得られること。回答に出典が付随し、規格に存在しない事項については推測ではなく「規格に記載なし」と明示されること。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>NFR-04</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>各工程閉幕の無作為抽出確認</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>各工程の閉幕時に無作為抽出による出典照合確認を組込む。事後是正ではなく工程閉幕の必須手順とする。本要件は事後検出のみに依存しない品質保証の要となる。</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>Accurate · Available</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>NFR-05</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>追跡可能性</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>任意の主張について、出典 PDF の該当頁および節を数秒で照合できる構造を提供する。ドメイン回答は三件 (spec / assumptions / examples)、章節回答は頁範囲付き Markdown、受控用語は C 符号で追跡可能とする。</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Attributable · Accurate</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>NFR-06</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>GAMP 5 / ALCOA+ 整合</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>本知識ベースの構築は、GAMP 5 (国際製薬技術協会 ISPE 発行) のリスク主導検証の考え方に整合する。具体的には、宣言された仕様、実行された確認、独立した審査、文書化された不整合追跡を備える。ただし、GAMP 5 への正式分類取得または ALCOA+ への公式認証取得は本範囲外とする。</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>BR-04</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>組内および他組への展開</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>本知識ベースが、統合 G 内のメンバー全員が同等に利用可能であり、将来的に関連業務組への展開も可能な形で構築されていること。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1901,131 +2124,162 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>5_制約条件</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>5_機能要件</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>制約 ID</t>
+          <t>機能要件 ID</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>種別</t>
+          <t>機能項目</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>制約内容</t>
+          <t>業務要件との対応</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>機能内容</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>C-01</t>
+          <t>FR-01</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>規格優先性</t>
+          <t>規格体系参照機能</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>本知識ベースの記述と CDISC 公式刊行物の記述に差異が見られた場合は、公式刊行物が優先される。規制当局への提出時の権威源は SDTMIG、SDTM Model、Controlled Terminology の各公式刊行物である。</t>
+          <t>BR-01</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>SDTM 規格の構造 (Domain、変数、章節、Controlled Terminology) を体系化して提供し、業務担当者が必要箇所を直接参照可能とする。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>C-02</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>規制範囲外</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="inlineStr">
-        <is>
-          <t>本知識ベースは、米国 21 CFR Part 11 または PMDA が想定する電子記録および電子署名要件を充足する電磁的記録の代替ではない。組織標準作業手順書が当該電子記録を規定する場合、その規定が優先される。</t>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>FR-02</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>出典追跡機能</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>BR-02</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>本知識ベース内の各記述に対し、公式刊行物の該当頁または節への追跡経路を保持する。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>C-03</t>
+          <t>FR-03</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>著作権</t>
+          <t>AI プラットフォーム連携機能</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>SDTM、SDTMIG、CDISC Controlled Terminology の各規格および原刊行物の著作権は CDISC が保持する。本リポジトリは原刊行物そのものを再配布せず、業務利用しやすい形に再構成した派生著作物のみを CC BY 4.0 ライセンスで配布する。原刊行物の入手は CDISC Library 経由で利用者が個別に行う。</t>
+          <t>BR-03</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>複数の主要 AI プラットフォームに対し本知識ベースを連携可能とし、平台経由の質問応答時に本知識ベースを参照源とする。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>C-04</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>機能限界</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>本知識ベースは、大規模な受控用語コードリストの完全展開および外部実時間検索の組込みを範囲外とする。これら個別事項の詳細は別途配布される技術文書 KNOWN_LIMITATIONS を参照する。</t>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>FR-04</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>多面検索機能</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>BR-01</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Domain 名、変数名、コントロールド・ターミノロジー用語名、C コード等による多面検索を提供する。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>C-05</t>
+          <t>FR-05</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>機密区分</t>
+          <t>共有参照経路提供機能</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>本知識ベースおよび関連納品文書の機密区分は公開可レベルとする。CDISC 規格自体が公開資料であり、これらに個人情報および組織機密情報を含めない。</t>
+          <t>BR-04</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>組内全員が同等にアクセス可能な参照経路 (社内共有形式およびネットワーク経由参照) を提供する。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -2044,117 +2298,117 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>6_前提条件</t>
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>6_非機能要件</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>前提 ID</t>
+          <t>非機能要件 ID</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>種別</t>
+          <t>観点</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>前提内容</t>
+          <t>要件内容</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>P-01</t>
+          <t>NFR-01</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>一次資料利用可能性</t>
+          <t>完全性</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>受信者は、必要に応じて CDISC 公式刊行物 4 件 (SDTMIG v3.4 PDF / SDTM Model v2.0 PDF / SDTMIG xlsx v3.4 / Controlled Terminology xlsx 2024 年版) を CDISC Library 経由で参照可能であることを前提とする。</t>
+          <t>本知識ベースは SDTM 規格の業務参照に必要な範囲を完全に網羅する。プレースホルダ (TBD 等) は完成版に残さない。規格対応部分に対する網羅率を定量化して提示する。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
-        <is>
-          <t>P-02</t>
-        </is>
-      </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>読者背景</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="inlineStr">
-        <is>
-          <t>受信者は IT 分野および医療データ分野の双方に知見を有する実務担当者であることを前提とする。基本的な臨床試験用語、Excel および Markdown の基本操作、業務系規格への抵抗のなさを想定する。</t>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>NFR-02</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>追跡可能性</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>本知識ベースの任意の記述について、公式刊行物の該当頁・節への追跡を業務担当者が独立に実施可能であること。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>P-03</t>
+          <t>NFR-03</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>概念整理</t>
+          <t>検索性能</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>受信者は SDTMIG v3.4 が SDTM Model v2.0 の実装ガイドである関係性を理解していることを前提とする。SDTM Model v2.0 は概念モデル (観察クラス、変数役割、ドメイン分類体系) を規定し、SDTMIG v3.4 はこれを前提として各ドメインの具体実装 (変数名、ラベル、Core 区分、業務上の前提、実装例) を規定する。</t>
+          <t>一般的な業務環境において、任意の参照対象に対する到達時間が数十秒以内であること。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>P-04</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>受控用語体系</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>受信者は CDISC 受控用語の C 符号体系 (例: C66731) を理解しており、米国国立がん研究所 EVS Browser (NCI EVS Browser) を用いた符号照合が可能であることを前提とする。</t>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>NFR-04</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>規制適合範囲の明示</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>本知識ベースが、米国 21 CFR Part 11 または PMDA 電子記録・電子署名指針が要求する電磁的記録の代替ではないこと、および変換業務最終成果物 (SDTM データセット) に対する規制対応は別途必要であることを、利用者が誤認しないよう本知識ベース内に明示する。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>P-05</t>
+          <t>NFR-05</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>確認根拠資料保管</t>
+          <t>規格優先性の明示</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>本知識ベースの構築過程で生成した確認根拠資料は、再監査可能な形式で組織内に保管されていることを前提とする。各処理単位の独立確認結果、覆盖率報告、無作為抽出確認記録を含む。</t>
+          <t>本知識ベースの記述と公式刊行物の記述に差異が見られた場合は公式刊行物が優先されることを、本知識ベース内に明示する。</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2419,7 @@
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
   <headerFooter>
-    <oddHeader>&amp;L要件定義書&amp;Cv1.0&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
+    <oddHeader>&amp;L要件定義書&amp;Cv1.1-draft&amp;R第 &amp;P 頁 / 全 &amp;N 頁</oddHeader>
     <oddFooter>&amp;L作成日: 2026-04-29&amp;R機密区分: 公開</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>